<commit_message>
Build 52 walk sheet + the release row (number read off the finished build)
26 rows organised by the founder's own findings, so each thing they reported has a row that says
what to do and what they should see. The row to check hardest is the right edge on Net worth — it
was genuinely bent by 8 points and the test meant to catch it could not. Four rows are marked
Device-only because no test can reach them: largest text size, greyscale, reduce-motion and the
app-switcher, and the keyboard over a save button.

The sheet deliberately does not hard-code the build number in its walk rows — last cut was reported
as 50 when it was 51, because the number was read from version:get (which returns the LAST used
number) instead of off the finished build. EAS states this one on the build itself: 52.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5572,6 +5572,33 @@
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>BUILD 52 CUT (v1.1.0 build 52 — number read OFF the finished build, from commit ec8e487 on taxonomy-v1.0.7, PUSHED before the cut so it is reproducible from the remote) after the founder's explicit "cut the build" to a presented pre-build checklist. Gate satisfied in order: scope complete (59/59 tracker rows; 13 commits since build 51, all from the founder's same-day device findings), audits FINISHED (open-gaps ledger 9 of 9 closed), adversarial journey pass green (5 suites / 64 tests), then the checklist. Fresh gates at the cut: 1,522 tests green, tsc clean, UI-test gate passing, clean tree. Contents: the account-naming rule, square banners app-wide, one money size and the 8-point right-edge fix, a Sync-now that syncs, a dead connection that says so, cash-means-cash enforced where data arrives, the leftover-is-cash rule, deposits landing in cash, income no longer guessed onto holdings, activity newest-first, the retirement card speaking below 80%, measured volatility, sample-and-ask, and the rewritten odds info dot. Walk sheet: docs/FCC-core-55-70/build52-founder-walk-2026-08-11.xlsx (26 rows, organised by the founder's own findings).</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>Founder: "cut the build" (2026-08-11), replying to the pre-build checklist.</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-11)</t>
         </is>

</xml_diff>

<commit_message>
End-to-end walk: 10 common journeys + 10 edge cases
New suite src/__tests__/e2e_walk_2026_08_11.test.tsx drives real screens
and real controls, then checks the next surface. C1-C10 cover the
everyday journeys; E1-E10 cover empty state, totals that do not
reconcile in both directions, an underwater net worth, an uncomputable
plan, a person past their retirement age, a dead connection, a
money-market fund and colliding account names.

It found one real defect: the plan-answers screen spoke the verdict as
'Unlikely - 0 in 100' while Home, Net worth and the Plan hub say
'Unlikely - 0% odds of lasting to age 92'. It now calls the same shared
oddsLine() helper. Pinned by C6.

1565 tests green, tsc clean, UI gate passes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5896,6 +5896,33 @@
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Plan answers — the verdict speaks the ONE app-wide wording</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>FOUND BY THE END-TO-END WALK. Home, Net worth and the Plan hub all say "&lt;word&gt; — xx% odds of lasting to age abc", but the answers screen — the very screen a person lands on to fix their odds — said "&lt;word&gt; — 0 in 100" instead, with no age in it. Worse, the same screen switched wording between its own two states: its SAMPLE line already read "Sample: 84% odds of lasting to age 90". It now calls the same shared oddsLine() helper the other three screens call, so there is one sentence in one place. Pinned by test C6, which renders all three surfaces for one person and fails unless the sentences are identical.</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>Founder rule 2026-08-11: "Let's make sure we are using same language everywhere to convey same message — xx% odds of lasting to age abc" — the walk found the one screen that was not.</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-11)</t>
         </is>

</xml_diff>

<commit_message>
Plan-surface redesign brief for Claude Design
Ground truth dumped from the running app: the Plan tab plus all 12
screens it opens, both personas, real strings and numbers. Brief carries
the approved design language, the nav map, the two personas, the ten
problems to solve, the calculation facts, the constraints and the
deliverable list.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E113"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5925,6 +5925,33 @@
       <c r="E113" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Plan surface — redesign brief written for Claude Design</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>THE WHOLE PLAN SURFACE GOES OUT FOR REDESIGN BEFORE THE NEXT CUT. Brief saved at mockups/Plan-redesign-Aug-12/PLAN-REDESIGN-BRIEF-v1-2026-08-12.md. It carries: the app in one page; the approved design language that must hold (flat ledger, square banners, ONE right edge, dollar-first, plain English, the one odds wording, hide-balances, 44pt, 10.5pt type floor); the Plan tab and all 12 screens it opens, dumped from the RUNNING app with real strings and real numbers for a 58-year-old worker and a 72-year-old retiree; the entry points from Home and Net worth; the two personas with reconciling numbers; the ten problems to solve (four sandboxes, the hub as a shopping list, the cockpit duplicating Performance, worker-vs-retiree divergence, machinery showing in empty states, Sharpen as a chore list, no picture of the plan over time, two first-year withdrawal numbers, the dead-end Social Security screen for someone already claiming, no single read-back of the plan); the calculation facts they must not contradict; what they may not change; and the deliverable list with states. Three known inconsistencies flagged for them to design around: two verdict word-sets for one number (Holding vs Likely), the explainer saying 500 runs when the engine runs 400, and the explainer saying 2.5% inflation when the screen shows a live 3.2%.</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12: "Let's also redesign Plan and associated screens before next cut. Can you give me instruction to feed to claude design to help design those screens."</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan redesign brief v2: architecture settled
Two sections; the answers screen, the what-if sandbox, the read-only
drivers and the big-costs list merge into one; facts save while choices
commit; the outcome carries a computed target nest egg and the yearly
saving it needs; the impossible-required-saving state is a required
design. v1 kept and superseded.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5950,6 +5950,33 @@
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Plan surface — architecture settled; brief v2 written</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>FOUNDER SETTLED THE PLAN ARCHITECTURE; brief bumped to mockups/Plan-redesign-Aug-12/PLAN-REDESIGN-BRIEF-v2-2026-08-12.md (v1 kept, superseded). DECIDED: (1) the Plan tab is TWO sections — "Your retirement plan" and "Decisions you can make today" — with "When can I retire?" in section 1, because it is the retire-at input wearing a question mark. (2) Section 1 is ONE MERGED SCREEN: the three answer questions + the What-if sandbox + the read-only drivers + the big-one-time-costs list, every field prefilled from a default or a calculation, anything genuinely unknown LABELLED as missing with a way to add it. Retire-at default 65 and plan-to default 90 become VISIBLE and changeable (they are already the code defaults but were applied silently). Retirement spending gets ASKED plainly, prefilled from today's spending — the app currently derives it and then tells the person "you set it", which is not true. (3) NEW RULE — facts save, choices commit: age/spending/what-counts/big-costs save on the spot; retire-at, claim age and extra saving stay drafts until "Use as my plan". (4) The outcome is two figures plus a line: the odds sentence, a goal tracker against a TARGET NEST EGG, and the yearly saving needed. The target is COMPUTED (the pile that puts the odds at 80%, the Likely boundary), not typed — a typed number stays as an optional marked override — so the tracker and the gauge are one fact drawn twice and can never contradict each other. The required saving is shown against the tax-advantaged room the app already knows. (5) The IMPOSSIBLE-REQUIRED-SAVING state is a required design: when the honest number exceeds what the person earns, say it plainly then pivot to the three levers that move (retire later, spend less, claim later) — never "you have failed". (6) The outcome must stay visible on a long screen. (7) What-if is absorbed and deleted; Multi-goal, Roth, Social Security timing, required withdrawals and the stress test survive in section 2, each row earning its place by saying what it is worth in dollars or points.</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12, across three exchanges: the six retirement inputs + defaults 65/90; the two-section layout; then "combine plan answers and Try what-ifs into one screen… add a big one-time cost… reverse calculate the monthly/annual savings goal based on targeted retirement nest egg" — with my recommendation to DERIVE the target from the odds rather than take a typed number, accepted.</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-12)</t>
         </is>

</xml_diff>

<commit_message>
The odds lose the verdict word
'60% odds of lasting to age 90' - no word in front. Both rival word-sets
deleted (Likely/Uncertain/Unlikely and Holding/Watch closely/Running
short), which also closes the two-words-for-one-number inconsistency.
Seven surfaces plus the desktop sandbox and the spoken labels. The info
dot now explains the number instead of defining a word.

1565 tests green, tsc clean, UI gate passed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5977,6 +5977,33 @@
         </is>
       </c>
       <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>The odds — the verdict word is removed, app-wide</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>THE WORD IS GONE. The odds now read "60% odds of lasting to age 90" with nothing in front. Removed on all seven surfaces that showed it — Home, Net worth, Plan hub, Plan answers, Will it last, Cash flow, Multi-goal — plus the desktop sandbox and the spoken screen-reader labels. BOTH rival word-sets are deleted from the code (Likely/Uncertain/Unlikely and the retiree Holding/Watch closely/Running short), which also closes the inconsistency where one retiree at 100% read "Holding" on the Plan tab and "Likely" on Will-it-last. The Multi-goal row that read "Uncertain to Uncertain" is gone — the row above it already says 60% to 67%. The info dot no longer defines a word that does not exist: it now opens WHAT THE NUMBER MEANS and says plainly why no word sits beside the percentage. Tests rewritten to pin the ABSENCE of the words on every surface, and the cross-screen agreement pin now reads the accessibility labels (what a screen reader hears) instead of hunting for a word beside a number — a stronger pin, because it fails if a screen shows the number without saying what it is. Gates: 1565 tests green, tsc clean, UI gate passed.</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12: "let's not say Uncertain — 60% odds of lasting to age 90. uncertain and giving it 60% probability does not make sense. it should be either or. Let's remove uncertain." Applied to all three bands and both voices, not just the middle word — the same objection holds for "Likely — 85%", and keeping one word while dropping another would have been worse than either.</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-12)</t>
         </is>

</xml_diff>

<commit_message>
Review of the Claude Design Plan handoff
Adopts the two-gauge hero, FACT/DRAFT chips, the five states and the
worth-labelled decision rows. Five corrections before code: the verdict
word (deleted by founder ruling after the brief went out), a range claim
that contradicts what the engine computes, the home's growth in a blend
that excludes the home, June's slack row vs its own arithmetic, and a
74% sample where the app's is 84%.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6006,6 +6006,33 @@
       <c r="E116" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>Plan redesign — Claude Design handoff received and reviewed</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>HANDOFF IN (Plan-requirements.md + Plan.dc.html), reviewed against the code; review saved at mockups/Plan-redesign-Aug-12/HANDOFF-REVIEW-2026-08-12.md. ADOPTED as drawn: the two-gauge hero (odds left, assets-vs-target right, both dollar figures beneath, then the bridge sentence "add $38,000/yr for 7 years to reach your target and raise your odds to 80%"), FACT/DRAFT chips as the at-a-glance tell between a saved fact and a draft choice, all five states of the merged screen with a pinned outcome strip, the honest impossible-saving state with three levers, worth-labelled Section 2 rows, and the retiree paycheck variant in place of a target gauge. FIVE CORRECTIONS before code: (1) BLOCKING — the design puts the verdict word on every screen ("Uncertain — 60% odds…"); the founder deleted the word hours after the brief went out, so every such line loses its word and nothing else moves. Not the designer's error: brief v2 asked them to pick a word-set; the sequencing was mine. (2) The handoff calls the 31-87% range a confidence band on the estimate and forbids saying "your odds could be as low as 31%" — but our engine derives that band by re-running the whole simulation at 2 percentage points lower and higher assumed return, so it IS a market-outcome range; the shipped wording "across bad-to-good markets" is correct and theirs would be false. (3) It puts the home's 4.5% growth into the blended return of a portfolio that excludes the home. (4) June's "spend more" row says "+$1,600/mo room" where the handoff's own arithmetic gives $2,555 unused safe draw — $1,600 is what she IS using. (5) The empty-state sample shows 74%; the app's sample is 84%, used everywhere. NEW ENGINE WORK identified (does not exist today): the derived target solved backwards for 80% odds, the required annual saving, per-lever point deltas, goals/debt wired into the odds engine for Section 2 labels, and the draft-vs-committed state layer — with a performance risk when one stepper move triggers a target solve plus a saving solve plus three lever runs. OPEN QUESTION for the founder: the handoff puts the merged screen behind a link from the tab rather than inside it, so the tab is a summary and the inputs are one tap away — that decides whether a person can change their retire age without leaving the tab.</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12 handed over the Claude Design output for the Plan surface.</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12) · review by me</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan outcome block: one score, then arithmetic
PlanOutcome renders the odds gauge, then three money lines that subtract
to each other - On track for / Target nest egg / Short - then the bridge
sentence. Above the target the third line flips to 'More than you need'.
The impossible state states the number once and turns to real levers.

7 component tests; 1583 green, tsc clean, UI gate passed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6033,6 +6033,33 @@
       <c r="E117" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-12) · review by me</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Plan outcome — one score, then arithmetic (second gauge dropped)</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>BUILDING THE ENGINE KILLED THE SECOND GAUGE. src/domain/planning/target.ts solves the odds backwards: targetAtRetirement (the pot on day one of retirement that reaches 80% odds, by bisection on the same 400-path simulation), requiredAnnualSaving (a second solve on the real plan, returned as the EXTRA over what they already save), and leverDeltas (each lever a genuine re-run with one change; claiming later raises the CHECK by 8%/yr, and the lever is hidden entirely when there is no Social Security on file). 11 engine tests incl. a speed budget — the whole outcome block is 238ms. THE FINDING: run a struggling person through it and the design contradicts itself — 31% odds beside a target gauge reading 80% of the way. Deriving the target does NOT prevent this, because progress compares ONE future (the median) against a threshold while the odds count how many of 400 futures lasted; the spread is what separates them. Founder accepted the fix: the right-hand side stops being a rival percentage. Asked whether it should be a gauge, a bar or text, the answer is TEXT — any proportional shape IS a score, and the eye believes the shape even after the number is removed. So: ONE score (the odds gauge), then three money lines that subtract to each other — On track for / Target nest egg (founder's words, replacing "You'd need") / Short — with the shortfall bold, then the bridge sentence naming the yearly amount and how much fits in tax-advantaged room. Above 100% the third line flips to "More than you need", which a gauge could not have drawn. The impossible state says the honest number once and turns to the levers. Built as src/components/PlanOutcome.tsx with 7 tests (one-score pin, the arithmetic ties to the dollar, the ahead state, the bridge, the impossible state, hide-balances, and the nothing-computable state). Mock deviation logged: the handoff's illustrative 60% / $1.9M / $38,000 do not survive contact with the engine — Pat as specified is 81% with a $1.14M target.</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12: "I am on with $" (the dollar gap over a second percentage), then "from design perspective is it still gauge or bar or simple text?" → text, and "It should not be You'd need - it is the Target Nest Egg."</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan tab: two sections, inputs on the tab
Section 1 is the tab - outcome, facts, choices - with the draft layer at
tab level so a stepper moves the number above it live. Section 2 is the
decisions that remain. The what-if door, the 'When can I retire?' row and
the big-costs door are gone: all three now live in section 1.

Four defects found by walking the built screen and fixed: a
contradictory 'more than you need' beside 'adding X closes it', the
stale narrative pair claiming 'you set it', and the two duplicate doors.

1593 green, tsc clean, UI gate passed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6058,6 +6058,33 @@
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Plan tab rebuilt — two sections, inputs ON the tab</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>SECTION 1 IS THE TAB, not a link behind it (founder ruling: "inputs on the tab"). The Plan tab now reads: YOUR RETIREMENT PLAN band → the outcome (one score, then On track for / Target nest egg / Short, then the bridge sentence) → FACTS — SAVE AS YOU GO (age, monthly spending in retirement, what counts, big one-time costs) → CHOICES — TRY THEM, NOTHING CHANGES YET (retire at, plan to age, extra saving) → DECISIONS YOU CAN MAKE TODAY. The draft layer lives at the tab so a stepper moves the number above it live (walked: 55% → 62% on one press of Retire at, with the projection and target moving too); "Use as my plan" confirms and writes. FOUR DEFECTS FOUND BY WALKING THE BUILT SCREEN, all fixed before reporting: (1) the outcome printed "More than you need $74,845" beside "Adding $43,000 a year closes it" — the median can clear the target while the odds do not, so the gap line now stands down whenever its sign disagrees with the odds and the bridge speaks alone; (2) the old narrative pair ("You could retire at 65 with…" + "…if you retire at 65, and spend $5,200/mo — your planned spending, you set it") was deleted: it repeated what the block above now says, did not follow the draft, and claimed "you set it" of a figure the app had derived; (3) the "Try what-ifs — a sandbox" door removed — the steppers ARE the sandbox, sitting under the number they move, so four sandboxes became one; (4) "When can I retire?" and "What big costs are coming?" removed from the decision list — both now live in section 1, and three copies of one question is how it got confusing. Gates: 1593 green, tsc clean, UI gate passed.</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12: "inputs on the tab." then "continue".</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-12)</t>
         </is>

</xml_diff>

<commit_message>
Fold /plan-answers into the Plan tab
The separate screen and route are deleted. The tab now carries the
missing-answer and empty states the design drew: MISSING chips, choices
stood down, a dashed can't-compute box in place of the odds. Home and
Net worth deep-link to the tab with ?focus=. The three ways in came back
from the shared DOORS list - the fold had dropped them.

Every test that pinned the deleted screen moved onto the tab.
1592 green, tsc clean, UI gate passed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6085,6 +6085,33 @@
         </is>
       </c>
       <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>/plan-answers folded into the Plan tab — one component, two states</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>THE LAST DUPLICATE IS GONE. The separate /plan-answers screen and route are DELETED; the Plan tab now carries the two states the Claude Design handoff drew as "Section 1 — Missing Age" and "Section 1 — Empty Sample": the age/spending row wears an amber MISSING chip, the choice steppers stand down (nothing for a choice to change yet), and a dashed box replaces the odds — "Your odds — can't work them out yet. Add what you spend below." Home and Net worth now deep-link to /(tabs)/plan?focus=&lt;the missing answer&gt; instead of a second screen; the tab reads the focus param and marks that row. The three ways in (connect / import / by hand) came back from the shared DOORS list — the fold had dropped them, which would have left someone with no accounts no way to add one; a source-pin test caught it. The route guard entry was removed with the route, and every test that pinned the deleted screen was MOVED onto the tab rather than deleted, including the cross-surface sameness pin, which now reads the spoken labels so a screen that shows the number without saying what it is fails. Gates: 1592 green, tsc clean, UI gate passed.</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12, on my own flag that two components were doing one job: "which screen in this in the plan-dc-html?" then "yes" to folding it before the cut. The handoff already had it right — plan-answers was never a screen in the design, only two states of Section 1.</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-12)</t>
         </is>

</xml_diff>

<commit_message>
The target nest egg is yours, and the parameters become questions
Two founder rulings, mocked not built.

The target is typed, not derived. "What's your target nest egg?" is a fact
the person enters and it is marked as theirs; the app's own 80%-odds figure
becomes the suggestion offered when the field is blank. That reverses a line
in my own brief - "the target is computed, not typed" was my call, and the
audit then held the number to a definition the founder never chose.

The retirement parameters stop being labels. How old are you. When do you
want to retire. How long should the money last. What counts toward
retirement. What big one-time costs are coming. The same words have to land
on all four surfaces that ask them, or the screens disagree.

Mock: rich state, first day, and a before/after wording table.
Audit workbook gains the rulings and two new rows; changelog logged same day.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6141,6 +6141,33 @@
       <c r="E121" t="inlineStr">
         <is>
           <t>Audit by me — awaiting founder verdicts</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Plan — the target nest egg is the person's own, and the parameters become questions</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>TWO RULINGS. (1) THE TARGET IS TYPED, NOT DERIVED. It is 'Your target nest egg' / 'What's your target nest egg?' — a fact the person enters, marked as theirs. The app's own 80%-odds figure becomes the SUGGESTION offered when the field is left blank, never the headline. This reverses brief v2 §'The target is computed, not typed', which was my call, not the founder's. Consequence: the money block reads down to THEIR gap (target − on track for = short) and the saving sentence closes THAT gap; the odds stay a separate honest number, because a pile of money and the chance it survives being spent are different things. (2) THE RETIREMENT PARAMETERS ARE QUESTIONS, NOT LABELS — current age, target retirement age, plan-to age, nest egg / retirement assets: 'How old are you?', 'When do you want to retire?', 'How long should the money last?', 'What counts toward retirement?', 'What big one-time costs are coming?', 'How much extra can you save each month?'. Founder: 'These are simple to understand.' The same words must land on all FOUR surfaces that ask them (Plan tab · Retirement cockpit · What drives this? · What if I save more?) or the screens will disagree. MOCK FIRST: mockups/Plan-redesign-Aug-12/plan-questions-and-typed-target-v1-2026-08-12.html (rich state + first day + a before/after wording table). NOT BUILT — awaiting the founder's yes.</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12, answering my audit finding D1: 'Target nest egg is a number entered by the user based on what is their target' + 'you type it and call it Your target nest egg... We should not have these retirement parameters as simply parameters versus framing it as a question.' The audit had held the target to a definition the founder never chose.</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12) — mock awaiting approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The decision rows get an ordering rule, because there wasn't one
The founder asked what determines the order and the honest answer was
nothing - the rows are hard-coded in whatever sequence the lines sit in the
file, and the brief had just carried the order he typed them in. Same gap
as the destinations, in a different place.

Dated things go first because they expire, which extends the one principle
the app already had from a single card to the whole list. Everything else
holds a fixed order per lens, chosen by what is on the mind at that stage,
and it does not re-sort as balances move - a row a person learns the
position of stays there.

Ranking by size or impact was considered and rejected, with the reason
written down: rows changing position between visits with the person having
done nothing.

Two placements in that table are mine rather than his and are flagged as
such in the brief.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E125"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6247,6 +6247,33 @@
         </is>
       </c>
       <c r="E125" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Plan — the decision rows get an ordering RULE (there was none)</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>FOUND BY THE FOUNDER'S QUESTION 'what's the order and how are we determining it?': there was NO rule. The rows are hard-coded JSX in PlanHubScreen, one after another, in whatever order the lines happen to sit in the file — no sort, no rank. The only ordering principle anywhere in the app governs a single card (nextDecision(): 'a required withdrawal due this year outranks everything — it has a deadline'). Brief v3 had simply carried the order the founder typed them in, which was the same gap in a different place. NOW SETTLED: (1) ANYTHING DATED GOES FIRST, because it expires — extends the existing deadline principle from one card to the whole list. (2) EVERYTHING ELSE HOLDS A FIXED ORDER PER LENS, chosen by what is most on the mind at that stage of life, and it does NOT re-sort as balances move — a person who learns where a row sits finds it there next month. Working: Social Security (60+) · pay off the mortgage early · is converting to a Roth worth it. Drawing down: Social Security (only if not yet claiming) · can I spend more · which account do I draw from first · pay off the mortgage early · is converting to a Roth worth it. REJECTED, with the reason recorded: ranking by size or by impact, because rows would change position between visits with the person having done nothing — and because the mortgage row has no points figure until the engine work lands. (3) A row only takes a position IF IT APPLIES — the founder's own test: 'if I don't have mortgage will mortgage appear for me? if I don't have 401K, conversion of Roth is meaningless.' No: absent, never greyed out, never 'no mortgage on file'. Expect a SHORT list — Pat at 58 sees two rows, June at 72 sees three. FLAGGED AS MINE not his, for confirmation: Social Security at the top of both columns, and the mortgage row appearing for retirees at all. TO BUILD: this is a rule the code applies, never again a sequence someone types.</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-12: 'what's the order in which these appear on screen? And how we are determining that order?' then chose deadlines-first + relevance, and defined relevance by his own two examples (no mortgage, no 401k) which are about PRESENCE; the tie-break among rows that do appear was settled separately as stage-of-life.</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-12)</t>
         </is>

</xml_diff>

<commit_message>
The 80% promise is true now, not nearly true
Audit D1 and D2 were one cause with two symptoms. Both the suggested target
and the required yearly saving are found by hunting for the smallest amount
that clears 80% odds - then both rounded to the nearest step, which can land
back under the line the search had just cleared.

Rounding up instead. The suggested target went from $1,370,000 delivering
76% to $1,380,000 delivering 81%; the saving from $53,000 delivering 79% to
$53,500 delivering 81%.

The pin holds the promise rather than the implementation: holding the target
has to deliver at least 80%, and one step lower has to miss - so it cannot
be made to pass by simply inflating the number.

1618 green, tsc clean, UI gate passed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6330,6 +6330,33 @@
       <c r="E128" t="inlineStr">
         <is>
           <t>Me — no ruling required</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Plan — audit D1 + D2 FIXED: the 80% promise is true, not nearly true</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Founder ruling: 'round up'. ONE CAUSE, TWO SYMPTOMS, one word each. Both figures are found by hunting for the smallest amount that clears 80% odds, then rounded to read like human numbers — and both rounded to the NEAREST step, which can land back BELOW the line the search had just cleared. targetAtRetirement: Math.round(found/10_000) → Math.ceil. requiredAnnualSaving: Math.round(found/500) → Math.ceil. MEASURED BEFORE/AFTER on Pat: suggested target $1,370,000 delivering 76% → $1,380,000 delivering 81%; required saving $53,000 delivering 79% → $53,500 delivering 81%. Erring high was the deliberate choice — the sentence on screen says 'this gets you to 80%' and it must be true; the alternative (the exact solved figure, $1,374,382) is precise and unreadable as a target. NEW PIN src/domain/planning/target_rounding.test.ts holds the PROMISE not the implementation: holding the target must deliver ≥80%, saving the figure must deliver ≥80%, both must round to a whole step, and ONE STEP LOWER MUST MISS — so the fix cannot be gamed by simply inflating the numbers. Gates: 1618 green, tsc clean, UI gate passed. D1's original defect (the target is not the number that gives 80%) was already mostly settled by the typed-target ruling; this closes the residue — the SUGGESTION we offer when the field is left blank.</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, first item of a one-at-a-time walk back through the 2026-08-12 mock-match audit.</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
D4: the line that tells you what to do comes back
The suppression rule behind the finding dies with the typed target, but it
left two things.

The v3 handoff had dropped the closing sentence entirely - the hero states
a shortfall and then goes straight to the glance, offering nothing. It comes
back, measured against the person's own target rather than ours. And it has
to be solved rather than formula'd: the obvious annuity calculation gives
$82,000 for Pat and lands $22,000 short of the target it just promised to
reach, which is the D1/D2 defect wearing new clothes. Solved by search it is
$84,500, and one step lower misses.

And a state nobody has drawn: already past your own target. Type $800,000
and Pat is at 114% of target with 45% odds. Not a contradiction - two honest
answers to two different questions - but the screen has to carry it without
either looking like a bug.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6355,6 +6355,33 @@
         </is>
       </c>
       <c r="E129" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Plan — audit D4: the closing sentence comes back, and the over-target state gets designed</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Founder: 'good with recommendation'. The suppression rule behind D4 dies with the typed target. TWO THINGS IT LEFT: (1) THE MOST ACTIONABLE LINE ON THE SCREEN HAD VANISHED. The v3 handoff ends the hero at 'short $1,090,848' and goes straight to the glance — stating a problem, offering nothing. Restored to brief §3.1, now measured against THEIR target: 'Saving $84,500 a year over your 7 years to 65 reaches your target.' CRITICAL METHOD NOTE: it must be SOLVED, not formula'd. The obvious closed-form annuity calculation gives $82,000 for Pat and lands at $1,977,544 — $22,000 short of the target it just promised to reach, which is exactly the D1/D2 defect class in a new place. Measured properly by search: $84,500 lands at $2,021,514, one $500 step lower lands at $1,994,407 and misses. Added to §6 as engine work (today's solve targets 80% ODDS, a different question) and it carries the same pin shape as D1/D2. (2) NEW REQUIRED STATE 6 in brief §5: ALREADY PAST YOUR OWN TARGET, drawn nowhere. Not a rare case — type $800,000 and Pat is at 114% of target with 45% odds: a dial pegged past full beside a number under half. Not a contradiction, two honest answers to two different questions, and the screen must carry it without either looking like an error. Mirror case specified too: a $1,500,000 target is reached by saving $24,000/yr at 64% odds — you can hit your number exactly and still not be at 80%. Both go to Claude Design in the next pass.</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, item 4 of the one-at-a-time audit walk.</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
         </is>

</xml_diff>

<commit_message>
D5: the paycheck rows say whose money they are
June's paycheck on the Plan tab was two bare amounts with no names beside
them - a bill with the line items blanked out - sitting directly above a
note promising "the same paycheck as Home's card, one engine, one set of
numbers".

The screen asked the engine for a field that does not exist. Home, month
detail and the paycheck months list all ask for the right one, so the Plan
tab was the only wrong consumer of four and there was no class to sweep.

Pinned three ways, and the pin was checked against the original bug rather
than trusted: reverting the fix fails two of the three.

1621 green, tsc clean, UI gate passed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6382,6 +6382,33 @@
         </is>
       </c>
       <c r="E130" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Plan — audit D5 FIXED: the retirement paycheck rows say whose money they are</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Founder: 'fix it'. June's paycheck on the Plan tab rendered two bare amounts with NO NAMES beside them — a bill with the line items blanked out — directly above a note reading 'the same paycheck as Home's card, one engine, one set of numbers'. Cause: PlanHubScreen read g.label off each guaranteed-income row; the engine's field is g.source. Home's PaycheckCard, MonthDetailScreen and PaycheckMonthsScreen all read it correctly — the Plan tab was the ONLY one of four consumers that was wrong, so the class needed no sweep. One word. NEW PIN src/__tests__/paycheck_row_names.test.tsx: (1) the Plan tab names every guaranteed row, (2) it names them the same way Home does, rendered through the one shared engine, (3) a source GUARD so no screen reaches for .label on a guaranteed row again. THE PIN WAS VERIFIED TO BITE — the fix was reverted, 2 of the 3 tests failed, and it was restored (the Home comparison passes either way, correctly, since Home was never broken). Fixed in place rather than left for the redesign: a one-word change, and a nameless paycheck is exactly what a device walk would hit first. Gates: 1621 green, tsc clean, UI gate passed.</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, item 5 of the one-at-a-time audit walk — the first finding nothing had overtaken.</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
         </is>

</xml_diff>

<commit_message>
D8: a retiree is not reaching for a target
June was shown a target nest egg, a "more than you need $585,000", and four
lines later "~$2,336,000 to spare" - two spare figures measuring different
things, neither labelled as which. And she was being told there was nothing
more to put away, about a plan she stopped paying into when she retired.

A target is a will-I-get-there framing. Once you are drawing down the
question is whether this is covering you, and the paycheck answers that. We
adopted the reasoning when the handoff arrived and confirmed it again
yesterday; it had never been built.

Her screen now reads the odds, then one spare figure on the line that also
carries her withdrawal rate. The levers block stays for retirees, because
spending less and claiming later genuinely still move their odds.

Also aligned the harness fixture to June's pinned numbers, so the dumps and
the brief agree.

1628 green, tsc clean, UI gate passed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E134"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6490,6 +6490,33 @@
         </is>
       </c>
       <c r="E134" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Plan — audit D8 FIXED: a retiree is not reaching for a target</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Founder: 'fix it now'. The target rows and both target-reaching sentences now stand down for the retired lens. A target is a 'will I get there' framing; once you are drawing down the question is 'is this covering me', and the paycheck answers it. That was adopted when the Claude Design handoff arrived and reconfirmed 2026-08-13 when the founder chose the paycheck for June's second dial — it had simply never been built. BEFORE, measured on June's corrected numbers: 'On track for $985,000 · Target nest egg $400,000 · More than you need $585,000', then 'You've cleared the 80% mark — nothing more to put away to stay there', then four lines later '~$2,336,000 to spare'. TWO SPARE FIGURES on one screen measuring different things (today's money against a target pot; the median left at 94), neither labelled as which, and a woman who is not saving being told to put nothing more away. AFTER: the odds, then a single spare figure on the line that also carries her 1.9% withdrawal rate. The impossible-state levers block is deliberately KEPT for retirees — spending less and claiming later still move a retiree's odds, so that is not target framing. Pinned by 5 tests including one proving a working-lens person is unaffected. Converges with the redesign, whose June frames carry no target rows either. NOTED WHILE LOOKING, not part of D8: that same line still says 'within the safe range' — the banned-word sweep the founder approved (29 places, 14 files) is still pending. Gates: 1628 green, tsc clean, UI gate passed.</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, item 8 of the one-at-a-time audit walk.</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
         </is>

</xml_diff>

<commit_message>
View A groups by where screens are actually reached from
The founder went looking for Insights and Sharpen on Home and pointed out
they are not there. He is right - Home links to neither. The map's facts were
correct, but its structure lied: View A said "measured" and was grouped by
each screen's proposed home, so those two sat in a box headed Home. Same
defect I flagged in the handoff's gauges, where the needle disagreed with the
numeral - the eye believes the shape, not the small print.

It now groups by where a person actually finds a screen. Where that view and
the proposal disagree, the gap is the finding, and the caption says so.

The regrouping immediately shows something worth knowing: ten screens hang
off the hamburger menu alone.

Insights and Sharpen are recorded as agreed moves onto Home. Not built -
adding links to Home is a screen change, and mock-first applies.

1633 green, output stable.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6654,6 +6654,33 @@
       <c r="E140" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Screen map — View A regrouped by where screens are actually reached from; Insights + Sharpen agreed onto Home</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>FOUNDER FOUND A REAL FLAW IN MY DOCUMENT: 'the latest home screen in last build does not link to insights or sharpen your plan.' Verified in code — HomeScreen links to NEITHER. Insights is reachable only from the ☰ menu; Sharpen only from the Plan tab, will-it-last and an insight card. The map was not wrong on the facts (the door line under each box said so) but its STRUCTURE lied: View A was labelled 'as it is today — measured' and yet grouped by each screen's PROPOSED home, so Insights and Sharpen sat inside a box headed 'Home'. Same defect I flagged in the design handoff's gauges — a shape saying one thing while the small print says another, and the eye believes the shape. FIXED: View A now groups by WHERE A PERSON ACTUALLY FINDS IT, measured — the tab bar itself (5) · from Home (3) · from Net worth (5) · from Performance (3) · from Cash flow (3) · from Plan (6) · from the ☰ menu (10) · deeper in, from another screen (4) · only when the data offers it (4) · nowhere (5) · second routes and redirects (3). Where View A and the proposal disagree, THAT GAP IS THE FINDING, and the caption now says so. NEW THING THE REGROUPING REVEALS: TEN screens hang off the ☰ menu alone — Goals, Retirement, Settings, Education, Estate, Insurance, Tax organiser, Stress test, Expense, Insights. FOUNDER DECISION SAME MESSAGE: 'I do agree insights, and sharpen both belong on the home screen' — both recorded as agreed moves in the map (Insights: menu → Home; Sharpen: Plan → Home). NOT BUILT: adding links to Home is a screen change and the mock-first standing order applies. Count now reads 31 of 48 stay, 11 move, 6 await a ruling. Gates: 1633 green, tsc clean, UI gate passed, output stable across runs.</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, reading the map against the built Home screen.</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13) — Home change awaiting a mock</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The dials stay while you edit - shrunk, not dropped
The v3 handoff contradicted itself: the drawing removed both dials from
Pat's expanded frame while its own note said the dials never move. Checked
the file - collapsed has two, expanded has none. The founder ruled for the
note.

The reason matters more than the pixels. Watching the odds respond is the
entire point of putting the inputs on the tab rather than behind a link.
Nudge the retirement age with the dials gone and you are adjusting blind,
then scrolling back to find out what happened - a taller screen and a worse
one.

Recorded in the brief; four of the five handoff rulings left.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E148"/>
+  <dimension ref="A1:E149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6870,6 +6870,33 @@
       <c r="E148" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13) — closes on the next device walk</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Plan — the dials stay visible while the glance is open (shrunk, not dropped)</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Founder: 'agree - keep the dials and shrink them.' Settles a contradiction inside the Claude Design v3 handoff itself: the drawing removed BOTH dials from Pat's expanded frame, replacing them with a single line of text, while the accompanying requirements note stated the dials 'never move'. Verified against the file on disk — the collapsed frame carries 2 dials, the expanded frame carries 0. The founder ruled for the note. THE REASON MATTERS MORE THAN THE PIXELS: watching the odds respond is the entire point of putting the inputs on the tab instead of behind a link. A person nudges the retirement age in order to see what it does; with the dials gone they are adjusting numbers blind and then scrolling back up to find out what happened — a taller screen AND a worse one. So the dials shrink and stay, with the number being changed and the number it is being changed for on screen together. How small, and whether they pin or compress in place, left to the designer. Recorded in brief v3 §3.2 and struck off the handoff review's open list — four of its five rulings remain.</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, first of the five handoff-review rulings.</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop the link that went nowhere on the worst screen in the app
The bad-odds frame offered "try all three together", pointing at a sandbox
that was folded into this tab last week - the steppers are the sandbox now.
It was never built, only drawn, so nothing ships broken and no code changes.

Same shape as the mortgage row and the free-route rows: an arrow with
nothing behind it. This one just happened to sit where the person is in the
most trouble.

The idea survives in the brief. Trying two or three changes at once is a
real question, but the screen could only honour two of the three today,
since claiming later is not a stepper. Half-delivering there is worse than
offering one fewer thing - so if the redesign wants it, it has to honour all
three and say what it needs.

Three of the five handoff rulings left.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6895,6 +6895,33 @@
         </is>
       </c>
       <c r="E149" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Plan — the "try all three together" link is dropped from the bad-odds screen</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Founder agreed the recommendation. The v3 handoff ends its bad-odds frame with 'Try all three together — one sandbox ›', pointing at the what-if sandbox the founder folded into this tab on 2026-08-12 — the steppers ARE the sandbox now, so the link has no destination. VERIFIED IT WAS NEVER BUILT: the phrase appears nowhere in src/, only in the drawing, so nothing ships broken today and no code changes. Same defect class as the mortgage row and the three free-route rows — an arrow with nothing behind it — except this one sits on the screen where the person is already in the most trouble. THE IDEA IS KEPT, THE LINK IS NOT: 'what if I did two or three of these at once' is a real question, but today the screen could only honour two of the three, since retiring later and spending less are steppers while claiming Social Security at 70 is not. A link that half-delivers on the worst screen in the app is worse than one fewer option. Recorded in brief v3 §5 as something the redesign may offer properly, with the condition that it must honour all three and say what it needs. Struck off the handoff review — three of its five rulings remain.</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, second of the five handoff-review rulings.</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
         </is>

</xml_diff>

<commit_message>
The decisions list stays when an age is missing
The handoff hid it: "decisions are hidden until your odds can be computed."
The founder's own list is the argument against. Paying off a mortgage needs
a mortgage, not an age. Converting to a Roth needs pre-tax money, not an age.
Both work for someone who linked their accounts and skipped one question, and
hiding them leaves an empty section where two actionable things belong.

The rows that do need an age now remove themselves - Social Security between
60 and 70, the required withdrawal at 73. So show what applies and let the
rest stay away on its own.

The built app already behaves this way, so this is an instruction to the
designer rather than a code change. The locked "when can I retire?" row
stays, because that one genuinely cannot be answered - and a lock explains
itself where an empty section does not.

Four of the five handoff rulings closed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E151"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6949,6 +6949,33 @@
         </is>
       </c>
       <c r="E151" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Plan — the decisions list stays when an age is missing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Founder: 'i like your recommendation.' The v3 handoff ends its age-missing frame with 'Decisions are hidden until your odds can be computed.' Rejected, and the founder's own decision list is the proof: PAYING OFF THE MORTGAGE EARLY NEEDS A MORTGAGE, NOT AN AGE; CONVERTING TO A ROTH NEEDS PRE-TAX MONEY, NOT AN AGE. Both work for someone who has linked accounts and skipped one question, and hiding them leaves an empty section where two actionable things belong — against this app's own rule that an empty state is an on-ramp, never a dead end. The rows that genuinely need an age already remove themselves after today's other rulings: Social Security is gated 60-70, the required withdrawal 73+. VERIFIED THE BUILT APP ALREADY DOES THIS — the missing-age render shows a locked 'When can I retire? 🔒' plus the decisions that apply — so this is a brief instruction to the designer, not a code change. KEPT FROM THE HANDOFF'S INSTINCT: the locked row is right, because that question truly cannot be answered without an age. A lock explains itself; an empty section does not. The designer's counter-argument is recorded rather than dismissed: without odds a decision can only say what it is worth in dollars and years, not points — but the points figure is not wired for either row yet, so nothing is lost today, and dollars and years are the honest half. Four of the five handoff rulings are now closed.</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, fourth of the five handoff-review rulings.</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
         </is>

</xml_diff>

<commit_message>
Hide-balances: the odds stay, the target numeral dots, the arc remains
The founder's call, and not the one I recommended. I argued for hiding the
target dial outright - its percentage is built from two dollar figures and
the arc carries the same ratio the numeral does, so the shape leaks what the
dots conceal. He chose to keep the shape, knowing that.

Both the ruling and the reservation are in the brief, so whoever reads it
next sees the trade instead of rediscovering it.

One refinement offered rather than assumed: if the arc is all that is left,
it does not have to be precise. A coarse fill reads "about this far" and
gives a shoulder-surfer much less than a needle at exactly 45%. The designer
can take it or refuse it with a reason.

That closes all five handoff-review rulings.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6976,6 +6976,33 @@
         </is>
       </c>
       <c r="E152" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Plan — hide-balances: the odds stay, the target numeral dots, the arc remains (closes the handoff review)</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Founder: 'hide the number, keep the shape.' Under hide-balances the ODDS dial stays fully visible — '48% odds of lasting to age 90' is not money and gives nothing away. On the TARGET dial the numeral is replaced by dots while the arc still fills to where it would. MY RECOMMENDATION WAS DIFFERENT AND IS RECORDED RATHER THAN QUIETLY DROPPED: I argued for hiding that dial outright, because its percentage is built entirely from two dollar figures ($909,152 ÷ $2,000,000) and the arc conveys the same ratio the numeral does — so the shape leaks what the dots conceal, and a privacy switch that half works is worse than one that is predictable. The founder made an informed choice; the brief now carries both the ruling and the reservation, so the next person reading it can see the trade rather than rediscover it. A REFINEMENT OFFERED, NOT ASSUMED: if the arc is the only thing left, it need not be precise — filling to a coarse band reads 'about this far along' while giving a shoulder-surfer much less than a needle at exactly 45%. Left to the designer to accept or reject with a stated reason. Nothing to build today: the two-dial hero is the redesign, and the built screen's money already masks. THIS CLOSES ALL FIVE HANDOFF-REVIEW RULINGS.</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13, fifth and last of the handoff-review rulings.</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
         </is>

</xml_diff>

<commit_message>
One named source of truth for the Claude Design handoffs
Four folders of deliveries had piled up outside the app, every one named
after net worth because that was the first screen drawn - though they now
hold Performance and Plan too. Compared byte for byte, three of the four
contain nothing unique except one file: the superseded v2 Plan drawing.

The latest is renamed to say what it is and when it arrived, and it sorts
to the top. Nothing deleted - the v2 drawing is a real earlier version and
the mock-first rule keeps those.

The v3 originals being on disk let me re-check the review against them
instead of the chat copies it was written from. They are clean, and B1 is
confirmed to the decimal: needles at 56.3 / 97.4 / 64.5 / 4.6 percent under
printed values of 48 / 100 / 84 / 12, arcs correct behind them. The warning
that the review might be reporting on mangled copies comes off.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E153"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7003,6 +7003,33 @@
         </is>
       </c>
       <c r="E153" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Claude Design handoffs — one named source of truth</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Four sub-folders of Claude Design deliveries had accumulated outside the app, all named after net worth because that was the first screen drawn, though they now also hold the Performance and Plan handoffs. A byte-for-byte comparison showed three of the four contain nothing unique except a single file — the superseded v2 Plan drawing. Founder: rename the latest so the single source of truth is obvious. Now '00-CURRENT-handoff-Net-worth-Performance-Plan-2026-08-13' — it names all three screens it holds, carries its delivery date, and sorts to the top of the folder. Nothing was deleted: the older copies stay where they are, and the v2 Plan drawing is a genuine superseded version that the mock-first rule says must be kept. The v3 originals are now ON DISK and the handoff review was re-checked against them rather than the chat copies it was first written from: the files are clean (no character corruption) and finding B1 is confirmed to the decimal — the six gauge needles point at 56.3%, 97.4%, 64.5% and 4.6% beneath printed values of 48%, 100%, 84% and 12%, while the arcs behind them are correct at 45.2% and 13.3%. The review's warning that it might be reporting on corrupted copies is lifted.</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-13: 'rename the latest folder that way we know what is single source of truth'.</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-13)</t>
         </is>

</xml_diff>

<commit_message>
Both briefs made sending-ready, and the two-version card approved
The founder approved the wording, so the 60-to-61 card is settled.

The Plan brief now opens its lessons section with a pointer to the handoff
review and leads on the defect worth fixing first - six needles pointing at
the wrong number over correct arcs, which we ask to be fixed with an angle
formula rather than placed coordinates. It also marks which two review items
are ours rather than the designer's, and asks for all three people.

The Home brief is welded to the Plan brief. Same people, one set of figures,
taken rather than re-derived - the last round went wrong precisely because a
persona wore someone else's numbers. It asks for a Ray frame, since his
"what needs you" block carries a card Pat's never shows, which is how that
block proves it reads the person instead of printing a list. The
hide-balances ruling travels across with it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E156"/>
+  <dimension ref="A1:E157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7086,6 +7086,33 @@
       <c r="E156" t="inlineStr">
         <is>
           <t>Founder ruling 2026-08-13 (window); wording AWAITING founder confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Social Security card — the 60-to-61 wording APPROVED, and both briefs made sending-ready</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Founder: 'yes, I like the text.' The two-version card is approved and live. At 60 and 61: 'Your Social Security decision is coming up — you can first claim at 62, and every year you wait after that raises the check, up to 70. Worth deciding before it arrives.' From 62 onward the existing 'window is open' wording is unchanged. Both open the same screen. The changelog row logged earlier today as AWAITING founder confirmation is now settled. BRIEFS PREPARED TO SEND: the Plan brief now opens its 'what went wrong' section with a pointer to the handoff review and leads on the defect to fix first — all six gauge needles point at the wrong number (56/97/65/5 percent beneath printed 48/100/84/12) while the arcs behind them are correct, so we are asking for the angle formula rather than placed coordinates; it also marks the two review items that are ours rather than the designer's, and its deliverables now call for all three people. The Home brief is welded to the Plan brief so the same person cannot carry different figures on two screens: it takes every dollar from the Plan brief's persona section rather than re-deriving, asks for a Ray frame because his 'what needs you' block carries a card Pat's never shows, quotes the approved Social Security wording by age band, and now carries the hide-balances ruling across from the Plan surface with the reservation and the coarse-fill refinement stated.</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Closes the last wording gate; both briefs are now complete and internally consistent with each other.</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-13)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Spend-more: the odds beside the control must be live, and $5,600 must say what it is
The founder read June's row and asked what the $5,600 meant. Two defects.

"Held at odds of 80%" explains how the $2,555 was calculated. The brief puts
it on that number; the handoff moved it onto the running total, where it is
false everywhere except the far end. At rest June is at 100 percent - so as
drawn the screen prints 80 beneath a dial reading 100 for the same plan.

Measured, her curve is 100, 100, 100, 97, 90, 80. Which means her first
$1,000 a month costs her nothing - a far better answer than a static 80, and
the actual thing she opened the row to find out.

And $5,600 at zero extra is just what she spends today. An arrow pointing at
it reads as the result of a decision she has not made.

Brief §3.5 tightened, B7 logged, the whole curve pinned so a build cannot
reintroduce a fixed number.

1669 green, tsc clean.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E160"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7192,6 +7192,33 @@
         </is>
       </c>
       <c r="E160" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Plan · spend-more — the odds beside the control must be LIVE; $5,600 must say what it is</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Founder read June's spend-more row and asked what the $5,600 meant. Two defects in one line, both now written into brief §3.5 and logged as blocker B7 in the handoff review. FIRST, THE ODDS ARE WRONG AT THE DEFAULT AND CONTRADICT THE SAME SCREEN. The phrase 'held at odds of 80%' explains how the $2,555 was CALCULATED — the largest extra draw that still holds an 80% floor — and the brief attaches it to that figure. The handoff moved it onto the running total, where it is false everywhere except the far end. Measured on the engine: at $0 extra June is at 100%, still 100% at $500 and $1,000 extra, then 97% at $1,500, 90% at $2,000, and 80% only at the $2,555 maximum. As drawn, the screen would print 80% directly beneath a dial reading 100% for the identical plan — that reads as a broken app, not a nuance. The odds beside a live control must themselves be live, which is brief §6.1 (odds are only ever an output) applied to a stepper. The real curve is also a better answer than the static one: her first $1,000 a month costs her nothing, which is exactly what she came to that row to find out. SECOND, $5,600 IS UNLABELLED. At zero extra it is simply what she spends today, but an arrow pointing at it reads as the result of a decision she has not made; it needs naming at rest and becomes a '→ … in total' only once the control moves. The brief also now requires one sentence linking draw and spend — her guaranteed $4,000 does not change, so every extra dollar spent is an extra dollar drawn. Whole curve pinned in src/__tests__/june_numbers_probe.test.ts so the build cannot reintroduce a static odds figure. Nothing to build today: this control is the redesign, not shipped code.</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Founder-found 2026-08-14 reading the design; a wrong number beside a live control is the worst place for one.</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-14)</t>
         </is>

</xml_diff>

<commit_message>
Build 53 cut: the Plan redesign and the mortgage engine work
Founder gave the literal "cut the build" to the presented checklist. Gates
re-run fresh at the moment of the cut rather than carried over: clean tree,
typecheck clean, 1796 green, quality gate passing, screen map regenerated.

Last used iOS build number read off EAS as 52, so this is 53.

The engine change is the thing to check on device. It lets a loan payment
end, which raises the odds for anyone whose mortgage finishes inside their
plan - a group whose odds have been pessimistic with nothing on screen saying
so.

Four defects were found and fixed before the cut by the build audit and the
adversarial pass, three of them on day one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7759,6 +7759,33 @@
         </is>
       </c>
       <c r="E181" t="inlineStr">
+        <is>
+          <t>Founder (chat 2026-08-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>BUILD 53 CUT — v1.1.0 #53, the Plan redesign and the mortgage engine work</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Founder said the literal 'cut the build' to the presented checklist, which is the only thing that counts under the release gate. GATES RE-RUN FRESH AT THE MOMENT OF THE CUT, not carried over from earlier in the session: clean working tree on taxonomy-v1.0.7 at 263f741, typecheck clean, 1796 tests green, quality gate passing, screen map regenerated with no new orphans. Last used iOS build number read off EAS as 52, so this is 53. WHAT SHIPS: the typed target nest egg end to end (the founder's first correction of this redesign, and until now the app derived a figure and labelled it as theirs); the second dial; the closing sentence that projects rather than promises and explains that growth does almost half the work; three sub-tabs with Goals and Prepare landings; the mortgage-versus-Treasury comparison in both directions with the retirement consequence attached as two real simulation runs; 'Can I spend more?' in plain English with every stepper position a live run; the Social Security claim row answering in place; day one showing all seven questions with our assumptions labelled as ours; and the engine change that lets a loan payment END — which raises the odds for anyone whose mortgage finishes inside their plan, a group whose odds have been pessimistic with no screen saying so. FOUR DEFECTS WERE FOUND AND FIXED BEFORE THE CUT by the two audits, three of them on day one — the first screen anyone sees. KNOWN AND GOING IN WITH IT: Claude Design still owes five corrections, so their drawing and the app will differ until that lands; what shipped uses the correct numbers, not the wrong ones in their file. NEXT: verify TestFlight arrival, then a device walk — the engine change is the thing to check, because it moves real numbers.</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Founder 2026-08-14 explicit 'cut the build' to the pre-build checklist.</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-14)</t>
         </is>

</xml_diff>

<commit_message>
Build 53 finished and submitted, verified on the build object
Status FINISHED read off the build record rather than trusted from the CLI
output, from commit 263f741. Apple confirmed the upload and it is in
processing.

The auto-submit held this time. It has died with the session before, since it
is driven from the command line, and had to be rescued with eas submit
--latest. Not needed here.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-detailed-design-v1.3-2026-07-19.xlsx
@@ -2867,7 +2867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E182"/>
+  <dimension ref="A1:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7788,6 +7788,33 @@
       <c r="E182" t="inlineStr">
         <is>
           <t>Founder (chat 2026-08-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>BUILD 53 FINISHED and SUBMITTED — verified on the build object, not from the log</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>v1.1.0 build 53, status FINISHED, read off the build record rather than trusted from CLI output: build id a75fe656-3e88-4fbf-8a51-bdb5b4ecf1c3, from commit 263f741, started 7:49pm and finished 7:55pm. Apple confirmed the upload — 'Submitted your app to Apple App Store Connect' — and it is now in Apple's processing, which usually takes five to ten minutes before it appears in TestFlight. NOTE FOR NEXT TIME: the auto-submit HELD this session. It has died with the session before (it is driven from the command line, so killing the session kills it) and had to be rescued with 'eas submit --latest'. That did not happen here; it completed inside the same run. THE DEVICE WALK SHOULD LEAD WITH THE ENGINE CHANGE, because it moves real numbers: a loan payment now stops when the loan does, so anyone whose mortgage finishes inside their plan will see HIGHER odds than before. Their odds have been pessimistic and nothing on screen said so. If the founder's odds jump and it feels wrong, that is the first thing to report. Also worth walking: the target nest egg is now his to type with our figure offered and labelled as ours; day one shows all seven questions with assumptions tagged; and the mortgage decision now lives on Cash flow · Debt with the Treasury comparison.</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Verify status against the build object, never the log — the standing rule that caught a stale build number before.</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Claude (verified)</t>
         </is>
       </c>
     </row>

</xml_diff>